<commit_message>
Mise à jour automatique des prix Donner
</commit_message>
<xml_diff>
--- a/Prix_Donner_TTC.xlsx
+++ b/Prix_Donner_TTC.xlsx
@@ -2887,7 +2887,7 @@
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>【Piano + banc gratuit】Donner OURA R300 Professionnel Piano Numérique - Bois clair / Piano + Banc【Pack Officiel】</t>
+          <t>【Piano + banc gratuit】Donner OURA R300 Professionnel Piano Numérique - Bois clair / Piano</t>
         </is>
       </c>
       <c r="B246" t="n">
@@ -2897,7 +2897,7 @@
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>【Piano + banc gratuit】Donner OURA R300 Professionnel Piano Numérique - Bois clair / Piano</t>
+          <t>【Piano + banc gratuit】Donner OURA R300 Professionnel Piano Numérique - Bois clair / Piano + Banc【Pack Officiel】</t>
         </is>
       </c>
       <c r="B247" t="n">
@@ -2917,7 +2917,7 @@
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>【Piano + banc gratuit】Donner OURA R300 Professionnel Piano Numérique - Gris-brun / Piano + Banc【Pack Officiel】</t>
+          <t>【Piano + banc gratuit】Donner OURA R300 Professionnel Piano Numérique - Gris-brun / Piano</t>
         </is>
       </c>
       <c r="B249" t="n">
@@ -2927,7 +2927,7 @@
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>【Piano + banc gratuit】Donner OURA R300 Professionnel Piano Numérique - Gris-brun / Piano</t>
+          <t>【Piano + banc gratuit】Donner OURA R300 Professionnel Piano Numérique - Gris-brun / Piano + Banc【Pack Officiel】</t>
         </is>
       </c>
       <c r="B250" t="n">
@@ -4047,7 +4047,7 @@
     <row r="362">
       <c r="A362" t="inlineStr">
         <is>
-          <t>Donner HUSH X Guitare Électrique Sans Tête - Blanc / Guitare</t>
+          <t>Donner HUSH X Guitare Électrique Sans Tête - Sunburst / Guitare</t>
         </is>
       </c>
       <c r="B362" t="n">
@@ -4057,7 +4057,7 @@
     <row r="363">
       <c r="A363" t="inlineStr">
         <is>
-          <t>Donner HUSH X Guitare Électrique Sans Tête - Blanc / Guitare + Arena 2000 Pédale</t>
+          <t>Donner HUSH X Guitare Électrique Sans Tête - Sunburst / Guitare + Arena 2000 Pédale</t>
         </is>
       </c>
       <c r="B363" t="n">
@@ -4067,7 +4067,7 @@
     <row r="364">
       <c r="A364" t="inlineStr">
         <is>
-          <t>Donner HUSH X Guitare Électrique Sans Tête - Blanc / Guitare + JW Pédale</t>
+          <t>Donner HUSH X Guitare Électrique Sans Tête - Sunburst / Guitare + JW Pédale</t>
         </is>
       </c>
       <c r="B364" t="n">
@@ -4077,7 +4077,7 @@
     <row r="365">
       <c r="A365" t="inlineStr">
         <is>
-          <t>Donner HUSH X Guitare Électrique Sans Tête - Noir / Guitare</t>
+          <t>Donner HUSH X Guitare Électrique Sans Tête - Blanc / Guitare</t>
         </is>
       </c>
       <c r="B365" t="n">
@@ -4087,7 +4087,7 @@
     <row r="366">
       <c r="A366" t="inlineStr">
         <is>
-          <t>Donner HUSH X Guitare Électrique Sans Tête - Noir / Guitare + Arena 2000 Pédale</t>
+          <t>Donner HUSH X Guitare Électrique Sans Tête - Blanc / Guitare + Arena 2000 Pédale</t>
         </is>
       </c>
       <c r="B366" t="n">
@@ -4097,7 +4097,7 @@
     <row r="367">
       <c r="A367" t="inlineStr">
         <is>
-          <t>Donner HUSH X Guitare Électrique Sans Tête - Noir / Guitare + JW Pédale</t>
+          <t>Donner HUSH X Guitare Électrique Sans Tête - Blanc / Guitare + JW Pédale</t>
         </is>
       </c>
       <c r="B367" t="n">
@@ -4107,7 +4107,7 @@
     <row r="368">
       <c r="A368" t="inlineStr">
         <is>
-          <t>Donner HUSH X Guitare Électrique Sans Tête - Sunburst / Guitare</t>
+          <t>Donner HUSH X Guitare Électrique Sans Tête - Noir / Guitare</t>
         </is>
       </c>
       <c r="B368" t="n">
@@ -4117,7 +4117,7 @@
     <row r="369">
       <c r="A369" t="inlineStr">
         <is>
-          <t>Donner HUSH X Guitare Électrique Sans Tête - Sunburst / Guitare + Arena 2000 Pédale</t>
+          <t>Donner HUSH X Guitare Électrique Sans Tête - Noir / Guitare + Arena 2000 Pédale</t>
         </is>
       </c>
       <c r="B369" t="n">
@@ -4127,7 +4127,7 @@
     <row r="370">
       <c r="A370" t="inlineStr">
         <is>
-          <t>Donner HUSH X Guitare Électrique Sans Tête - Sunburst / Guitare + JW Pédale</t>
+          <t>Donner HUSH X Guitare Électrique Sans Tête - Noir / Guitare + JW Pédale</t>
         </is>
       </c>
       <c r="B370" t="n">

</xml_diff>